<commit_message>
Detail all 7 subsystem tracks + floor plan; add feasibility assay & BOM; sodium (CATL Naxtra) mass/energy update
</commit_message>
<xml_diff>
--- a/00_Admin_Budget_Schedule/House_BUS_Mass_Budget.xlsx
+++ b/00_Admin_Budget_Schedule/House_BUS_Mass_Budget.xlsx
@@ -270,7 +270,7 @@
     <t xml:space="preserve">Battery pack 300 kWh</t>
   </si>
   <si>
-    <t xml:space="preserve">modules+enclosure -&gt; structural sodium/blade</t>
+    <t xml:space="preserve">sodium-ion CTP/structural (CATL Naxtra ~175 Wh/kg, mass-prod 2025)</t>
   </si>
   <si>
     <t xml:space="preserve">Power electronics</t>
@@ -564,12 +564,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -577,7 +581,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -585,11 +589,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -597,11 +601,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -625,11 +629,11 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -641,11 +645,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -912,247 +916,247 @@
   <dimension ref="A1:D22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="40"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="5" t="n">
         <f aca="false">'Mass Budget'!$C$37</f>
         <v>18240</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="7" t="n">
+      <c r="B5" s="8" t="n">
         <f aca="false">'Mass Budget'!$C$38</f>
-        <v>12970</v>
-      </c>
-      <c r="C5" s="8" t="s">
+        <v>13270</v>
+      </c>
+      <c r="C5" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="10" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="10" t="n">
+      <c r="B6" s="11" t="n">
         <f aca="false">'Mass Budget'!$C$40</f>
-        <v>0.288925438596491</v>
-      </c>
-      <c r="C6" s="8"/>
-      <c r="D6" s="9" t="s">
+        <v>0.272478070175439</v>
+      </c>
+      <c r="C6" s="9"/>
+      <c r="D6" s="10" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="11" t="n">
+      <c r="B7" s="12" t="n">
         <f aca="false">Assumptions!$B$5*Assumptions!$B$6</f>
         <v>350</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="5"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="D7" s="6"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="11" t="n">
+      <c r="B8" s="12" t="n">
         <f aca="false">Assumptions!$B$7*Assumptions!$B$8</f>
         <v>417</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D8" s="5"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="D8" s="6"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="11" t="n">
+      <c r="B9" s="12" t="n">
         <f aca="false">Assumptions!$B$9</f>
         <v>500</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D9" s="5"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="D9" s="6"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="11" t="n">
+      <c r="B10" s="12" t="n">
         <f aca="false">Assumptions!$B$10</f>
         <v>500</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D10" s="5"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
+      <c r="D10" s="6"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="12" t="n">
+      <c r="B11" s="13" t="n">
         <f aca="false">SUM(B7:B10)</f>
         <v>1767</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="D11" s="9"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
+      <c r="D11" s="10"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="12" t="n">
+      <c r="B12" s="13" t="n">
         <f aca="false">'Mass Budget'!$C$38+B11</f>
-        <v>14737</v>
-      </c>
-      <c r="C12" s="8" t="s">
+        <v>15037</v>
+      </c>
+      <c r="C12" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="D12" s="9"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="D12" s="10"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="11" t="n">
+      <c r="B13" s="12" t="n">
         <f aca="false">Assumptions!$B$4</f>
         <v>19500</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D13" s="5"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="s">
+      <c r="D13" s="6"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="12" t="n">
+      <c r="B14" s="13" t="n">
         <f aca="false">B13-B12</f>
-        <v>4763</v>
-      </c>
-      <c r="C14" s="8" t="s">
+        <v>4463</v>
+      </c>
+      <c r="C14" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="D14" s="10" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="13" t="n">
+      <c r="B15" s="14" t="n">
         <f aca="false">B14/B13</f>
-        <v>0.24425641025641</v>
-      </c>
-      <c r="C15" s="3"/>
-      <c r="D15" s="5"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+        <v>0.228871794871795</v>
+      </c>
+      <c r="C15" s="4"/>
+      <c r="D15" s="6"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B16" s="11" t="n">
+      <c r="B16" s="12" t="n">
         <f aca="false">'Mass Budget'!$C$41</f>
-        <v>156.360832690825</v>
-      </c>
-      <c r="C16" s="3" t="s">
+        <v>156.21703089676</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="D16" s="6" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="11" t="n">
+      <c r="B17" s="12" t="n">
         <f aca="false">B12*(B16-Assumptions!$B$11)/(Assumptions!$B$12-Assumptions!$B$11)</f>
-        <v>7814.87900649851</v>
-      </c>
-      <c r="C17" s="3" t="s">
+        <v>7963.66901711702</v>
+      </c>
+      <c r="C17" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="D17" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B18" s="11" t="n">
+      <c r="B18" s="12" t="n">
         <f aca="false">B12-B17</f>
-        <v>6922.12099350149</v>
-      </c>
-      <c r="C18" s="3" t="s">
+        <v>7073.33098288298</v>
+      </c>
+      <c r="C18" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D18" s="5"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="s">
+      <c r="D18" s="6"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B20" s="14" t="str">
+      <c r="B20" s="15" t="str">
         <f aca="false">IF(B14&gt;=0,"Within GVWR by "&amp;TEXT(B14,"#,##0")&amp;" lb","OVER GVWR by "&amp;TEXT(-B14,"#,##0")&amp;" lb")</f>
-        <v>Within GVWR by 4,763 lb</v>
-      </c>
-      <c r="C20" s="15"/>
-      <c r="D20" s="15"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="16" t="s">
+        <v>Within GVWR by 4,463 lb</v>
+      </c>
+      <c r="C20" s="16"/>
+      <c r="D20" s="16"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="17" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1175,149 +1179,149 @@
   <dimension ref="A1:D12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="40"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="17" t="n">
+      <c r="B4" s="18" t="n">
         <v>19500</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="17" t="n">
+      <c r="B5" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="17" t="n">
+      <c r="B6" s="18" t="n">
         <v>175</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="5"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="D6" s="6"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B7" s="17" t="n">
+      <c r="B7" s="18" t="n">
         <v>50</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="6" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="17" t="n">
+      <c r="B8" s="18" t="n">
         <v>8.34</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="17" t="n">
+      <c r="B9" s="18" t="n">
         <v>500</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="17" t="n">
+      <c r="B10" s="18" t="n">
         <v>500</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D10" s="5"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="D10" s="6"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="17" t="n">
+      <c r="B11" s="18" t="n">
         <v>45</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="6" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B12" s="17" t="n">
+      <c r="B12" s="18" t="n">
         <v>255</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D12" s="5"/>
+      <c r="D12" s="6"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1338,998 +1342,998 @@
   <dimension ref="A1:H44"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="13"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="3" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C3" s="17" t="n">
+      <c r="C3" s="18" t="n">
         <v>2500</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="E3" s="17" t="n">
+      <c r="E3" s="18" t="n">
         <v>1400</v>
       </c>
-      <c r="F3" s="18" t="n">
+      <c r="F3" s="19" t="n">
         <f aca="false">C3-E3</f>
         <v>1100</v>
       </c>
-      <c r="G3" s="17" t="n">
+      <c r="G3" s="18" t="n">
         <v>150</v>
       </c>
-      <c r="H3" s="18" t="n">
+      <c r="H3" s="19" t="n">
         <f aca="false">E3*G3</f>
         <v>210000</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="C4" s="17" t="n">
+      <c r="C4" s="18" t="n">
         <v>2500</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="E4" s="17" t="n">
+      <c r="E4" s="18" t="n">
         <v>1200</v>
       </c>
-      <c r="F4" s="18" t="n">
+      <c r="F4" s="19" t="n">
         <f aca="false">C4-E4</f>
         <v>1300</v>
       </c>
-      <c r="G4" s="17" t="n">
+      <c r="G4" s="18" t="n">
         <v>150</v>
       </c>
-      <c r="H4" s="18" t="n">
+      <c r="H4" s="19" t="n">
         <f aca="false">E4*G4</f>
         <v>180000</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="C5" s="17" t="n">
+      <c r="C5" s="18" t="n">
         <v>600</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="E5" s="17" t="n">
+      <c r="E5" s="18" t="n">
         <v>350</v>
       </c>
-      <c r="F5" s="18" t="n">
+      <c r="F5" s="19" t="n">
         <f aca="false">C5-E5</f>
         <v>250</v>
       </c>
-      <c r="G5" s="17" t="n">
+      <c r="G5" s="18" t="n">
         <v>150</v>
       </c>
-      <c r="H5" s="18" t="n">
+      <c r="H5" s="19" t="n">
         <f aca="false">E5*G5</f>
         <v>52500</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="C6" s="17" t="n">
+      <c r="C6" s="18" t="n">
         <v>350</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="E6" s="17" t="n">
+      <c r="E6" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="F6" s="18" t="n">
+      <c r="F6" s="19" t="n">
         <f aca="false">C6-E6</f>
         <v>50</v>
       </c>
-      <c r="G6" s="17" t="n">
+      <c r="G6" s="18" t="n">
         <v>150</v>
       </c>
-      <c r="H6" s="18" t="n">
+      <c r="H6" s="19" t="n">
         <f aca="false">E6*G6</f>
         <v>45000</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="C7" s="17" t="n">
+      <c r="C7" s="18" t="n">
         <v>350</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="E7" s="17" t="n">
+      <c r="E7" s="18" t="n">
         <v>180</v>
       </c>
-      <c r="F7" s="18" t="n">
+      <c r="F7" s="19" t="n">
         <f aca="false">C7-E7</f>
         <v>170</v>
       </c>
-      <c r="G7" s="17" t="n">
+      <c r="G7" s="18" t="n">
         <v>150</v>
       </c>
-      <c r="H7" s="18" t="n">
+      <c r="H7" s="19" t="n">
         <f aca="false">E7*G7</f>
         <v>27000</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="C8" s="17" t="n">
+      <c r="C8" s="18" t="n">
         <v>900</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="E8" s="17" t="n">
+      <c r="E8" s="18" t="n">
         <v>350</v>
       </c>
-      <c r="F8" s="18" t="n">
+      <c r="F8" s="19" t="n">
         <f aca="false">C8-E8</f>
         <v>550</v>
       </c>
-      <c r="G8" s="17" t="n">
+      <c r="G8" s="18" t="n">
         <v>160</v>
       </c>
-      <c r="H8" s="18" t="n">
+      <c r="H8" s="19" t="n">
         <f aca="false">E8*G8</f>
         <v>56000</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="C9" s="17" t="n">
+      <c r="C9" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="E9" s="17" t="n">
+      <c r="E9" s="18" t="n">
         <v>180</v>
       </c>
-      <c r="F9" s="18" t="n">
+      <c r="F9" s="19" t="n">
         <f aca="false">C9-E9</f>
         <v>120</v>
       </c>
-      <c r="G9" s="17" t="n">
+      <c r="G9" s="18" t="n">
         <v>150</v>
       </c>
-      <c r="H9" s="18" t="n">
+      <c r="H9" s="19" t="n">
         <f aca="false">E9*G9</f>
         <v>27000</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="C10" s="17" t="n">
+      <c r="C10" s="18" t="n">
         <v>1100</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="E10" s="17" t="n">
+      <c r="E10" s="18" t="n">
         <v>950</v>
       </c>
-      <c r="F10" s="18" t="n">
+      <c r="F10" s="19" t="n">
         <f aca="false">C10-E10</f>
         <v>150</v>
       </c>
-      <c r="G10" s="17" t="n">
+      <c r="G10" s="18" t="n">
         <v>250</v>
       </c>
-      <c r="H10" s="18" t="n">
+      <c r="H10" s="19" t="n">
         <f aca="false">E10*G10</f>
         <v>237500</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="C11" s="17" t="n">
+      <c r="C11" s="18" t="n">
         <v>600</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="E11" s="17" t="n">
+      <c r="E11" s="18" t="n">
         <v>500</v>
       </c>
-      <c r="F11" s="18" t="n">
+      <c r="F11" s="19" t="n">
         <f aca="false">C11-E11</f>
         <v>100</v>
       </c>
-      <c r="G11" s="17" t="n">
+      <c r="G11" s="18" t="n">
         <v>160</v>
       </c>
-      <c r="H11" s="18" t="n">
+      <c r="H11" s="19" t="n">
         <f aca="false">E11*G11</f>
         <v>80000</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="C12" s="17" t="n">
+      <c r="C12" s="18" t="n">
         <v>600</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="E12" s="17" t="n">
+      <c r="E12" s="18" t="n">
         <v>550</v>
       </c>
-      <c r="F12" s="18" t="n">
+      <c r="F12" s="19" t="n">
         <f aca="false">C12-E12</f>
         <v>50</v>
       </c>
-      <c r="G12" s="17" t="n">
+      <c r="G12" s="18" t="n">
         <v>150</v>
       </c>
-      <c r="H12" s="18" t="n">
+      <c r="H12" s="19" t="n">
         <f aca="false">E12*G12</f>
         <v>82500</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="C13" s="17" t="n">
+      <c r="C13" s="18" t="n">
         <v>350</v>
       </c>
-      <c r="D13" s="5"/>
-      <c r="E13" s="17" t="n">
+      <c r="D13" s="6"/>
+      <c r="E13" s="18" t="n">
         <v>320</v>
       </c>
-      <c r="F13" s="18" t="n">
+      <c r="F13" s="19" t="n">
         <f aca="false">C13-E13</f>
         <v>30</v>
       </c>
-      <c r="G13" s="17" t="n">
+      <c r="G13" s="18" t="n">
         <v>110</v>
       </c>
-      <c r="H13" s="18" t="n">
+      <c r="H13" s="19" t="n">
         <f aca="false">E13*G13</f>
         <v>35200</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="C14" s="17" t="n">
+      <c r="C14" s="18" t="n">
         <v>4000</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="E14" s="17" t="n">
-        <v>3480</v>
-      </c>
-      <c r="F14" s="18" t="n">
+      <c r="E14" s="18" t="n">
+        <v>3780</v>
+      </c>
+      <c r="F14" s="19" t="n">
         <f aca="false">C14-E14</f>
-        <v>520</v>
-      </c>
-      <c r="G14" s="17" t="n">
+        <v>220</v>
+      </c>
+      <c r="G14" s="18" t="n">
         <v>150</v>
       </c>
-      <c r="H14" s="18" t="n">
+      <c r="H14" s="19" t="n">
         <f aca="false">E14*G14</f>
-        <v>522000</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+        <v>567000</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="C15" s="17" t="n">
+      <c r="C15" s="18" t="n">
         <v>250</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="D15" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="E15" s="17" t="n">
+      <c r="E15" s="18" t="n">
         <v>200</v>
       </c>
-      <c r="F15" s="18" t="n">
+      <c r="F15" s="19" t="n">
         <f aca="false">C15-E15</f>
         <v>50</v>
       </c>
-      <c r="G15" s="17" t="n">
+      <c r="G15" s="18" t="n">
         <v>240</v>
       </c>
-      <c r="H15" s="18" t="n">
+      <c r="H15" s="19" t="n">
         <f aca="false">E15*G15</f>
         <v>48000</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="C16" s="17" t="n">
+      <c r="C16" s="18" t="n">
         <v>350</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="D16" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="E16" s="17" t="n">
+      <c r="E16" s="18" t="n">
         <v>180</v>
       </c>
-      <c r="F16" s="18" t="n">
+      <c r="F16" s="19" t="n">
         <f aca="false">C16-E16</f>
         <v>170</v>
       </c>
-      <c r="G16" s="17" t="n">
+      <c r="G16" s="18" t="n">
         <v>150</v>
       </c>
-      <c r="H16" s="18" t="n">
+      <c r="H16" s="19" t="n">
         <f aca="false">E16*G16</f>
         <v>27000</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="C17" s="17" t="n">
+      <c r="C17" s="18" t="n">
         <v>350</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="D17" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="E17" s="17" t="n">
+      <c r="E17" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="F17" s="18" t="n">
+      <c r="F17" s="19" t="n">
         <f aca="false">C17-E17</f>
         <v>50</v>
       </c>
-      <c r="G17" s="17" t="n">
+      <c r="G17" s="18" t="n">
         <v>150</v>
       </c>
-      <c r="H17" s="18" t="n">
+      <c r="H17" s="19" t="n">
         <f aca="false">E17*G17</f>
         <v>45000</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="C18" s="17" t="n">
+      <c r="C18" s="18" t="n">
         <v>120</v>
       </c>
-      <c r="D18" s="5"/>
-      <c r="E18" s="17" t="n">
+      <c r="D18" s="6"/>
+      <c r="E18" s="18" t="n">
         <v>100</v>
       </c>
-      <c r="F18" s="18" t="n">
+      <c r="F18" s="19" t="n">
         <f aca="false">C18-E18</f>
         <v>20</v>
       </c>
-      <c r="G18" s="17" t="n">
+      <c r="G18" s="18" t="n">
         <v>200</v>
       </c>
-      <c r="H18" s="18" t="n">
+      <c r="H18" s="19" t="n">
         <f aca="false">E18*G18</f>
         <v>20000</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="C19" s="17" t="n">
+      <c r="C19" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="D19" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="E19" s="17" t="n">
+      <c r="E19" s="18" t="n">
         <v>280</v>
       </c>
-      <c r="F19" s="18" t="n">
+      <c r="F19" s="19" t="n">
         <f aca="false">C19-E19</f>
         <v>20</v>
       </c>
-      <c r="G19" s="17" t="n">
+      <c r="G19" s="18" t="n">
         <v>100</v>
       </c>
-      <c r="H19" s="18" t="n">
+      <c r="H19" s="19" t="n">
         <f aca="false">E19*G19</f>
         <v>28000</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="C20" s="17" t="n">
+      <c r="C20" s="18" t="n">
         <v>250</v>
       </c>
-      <c r="D20" s="5"/>
-      <c r="E20" s="17" t="n">
+      <c r="D20" s="6"/>
+      <c r="E20" s="18" t="n">
         <v>200</v>
       </c>
-      <c r="F20" s="18" t="n">
+      <c r="F20" s="19" t="n">
         <f aca="false">C20-E20</f>
         <v>50</v>
       </c>
-      <c r="G20" s="17" t="n">
+      <c r="G20" s="18" t="n">
         <v>150</v>
       </c>
-      <c r="H20" s="18" t="n">
+      <c r="H20" s="19" t="n">
         <f aca="false">E20*G20</f>
         <v>30000</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="C21" s="17" t="n">
+      <c r="C21" s="18" t="n">
         <v>200</v>
       </c>
-      <c r="D21" s="5"/>
-      <c r="E21" s="17" t="n">
+      <c r="D21" s="6"/>
+      <c r="E21" s="18" t="n">
         <v>180</v>
       </c>
-      <c r="F21" s="18" t="n">
+      <c r="F21" s="19" t="n">
         <f aca="false">C21-E21</f>
         <v>20</v>
       </c>
-      <c r="G21" s="17" t="n">
+      <c r="G21" s="18" t="n">
         <v>110</v>
       </c>
-      <c r="H21" s="18" t="n">
+      <c r="H21" s="19" t="n">
         <f aca="false">E21*G21</f>
         <v>19800</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="C22" s="17" t="n">
+      <c r="C22" s="18" t="n">
         <v>150</v>
       </c>
-      <c r="D22" s="5"/>
-      <c r="E22" s="17" t="n">
+      <c r="D22" s="6"/>
+      <c r="E22" s="18" t="n">
         <v>120</v>
       </c>
-      <c r="F22" s="18" t="n">
+      <c r="F22" s="19" t="n">
         <f aca="false">C22-E22</f>
         <v>30</v>
       </c>
-      <c r="G22" s="17" t="n">
+      <c r="G22" s="18" t="n">
         <v>120</v>
       </c>
-      <c r="H22" s="18" t="n">
+      <c r="H22" s="19" t="n">
         <f aca="false">E22*G22</f>
         <v>14400</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="C23" s="17" t="n">
+      <c r="C23" s="18" t="n">
         <v>250</v>
       </c>
-      <c r="D23" s="5" t="s">
+      <c r="D23" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="E23" s="17" t="n">
+      <c r="E23" s="18" t="n">
         <v>200</v>
       </c>
-      <c r="F23" s="18" t="n">
+      <c r="F23" s="19" t="n">
         <f aca="false">C23-E23</f>
         <v>50</v>
       </c>
-      <c r="G23" s="17" t="n">
+      <c r="G23" s="18" t="n">
         <v>130</v>
       </c>
-      <c r="H23" s="18" t="n">
+      <c r="H23" s="19" t="n">
         <f aca="false">E23*G23</f>
         <v>26000</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C24" s="17" t="n">
+      <c r="C24" s="18" t="n">
         <v>90</v>
       </c>
-      <c r="D24" s="5"/>
-      <c r="E24" s="17" t="n">
+      <c r="D24" s="6"/>
+      <c r="E24" s="18" t="n">
         <v>60</v>
       </c>
-      <c r="F24" s="18" t="n">
+      <c r="F24" s="19" t="n">
         <f aca="false">C24-E24</f>
         <v>30</v>
       </c>
-      <c r="G24" s="17" t="n">
+      <c r="G24" s="18" t="n">
         <v>200</v>
       </c>
-      <c r="H24" s="18" t="n">
+      <c r="H24" s="19" t="n">
         <f aca="false">E24*G24</f>
         <v>12000</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B25" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="C25" s="17" t="n">
+      <c r="C25" s="18" t="n">
         <v>60</v>
       </c>
-      <c r="D25" s="5"/>
-      <c r="E25" s="17" t="n">
+      <c r="D25" s="6"/>
+      <c r="E25" s="18" t="n">
         <v>50</v>
       </c>
-      <c r="F25" s="18" t="n">
+      <c r="F25" s="19" t="n">
         <f aca="false">C25-E25</f>
         <v>10</v>
       </c>
-      <c r="G25" s="17" t="n">
+      <c r="G25" s="18" t="n">
         <v>210</v>
       </c>
-      <c r="H25" s="18" t="n">
+      <c r="H25" s="19" t="n">
         <f aca="false">E25*G25</f>
         <v>10500</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="3" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B26" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="C26" s="17" t="n">
+      <c r="C26" s="18" t="n">
         <v>120</v>
       </c>
-      <c r="D26" s="5"/>
-      <c r="E26" s="17" t="n">
+      <c r="D26" s="6"/>
+      <c r="E26" s="18" t="n">
         <v>90</v>
       </c>
-      <c r="F26" s="18" t="n">
+      <c r="F26" s="19" t="n">
         <f aca="false">C26-E26</f>
         <v>30</v>
       </c>
-      <c r="G26" s="17" t="n">
+      <c r="G26" s="18" t="n">
         <v>160</v>
       </c>
-      <c r="H26" s="18" t="n">
+      <c r="H26" s="19" t="n">
         <f aca="false">E26*G26</f>
         <v>14400</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="3" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C27" s="17" t="n">
+      <c r="C27" s="18" t="n">
         <v>200</v>
       </c>
-      <c r="D27" s="5" t="s">
+      <c r="D27" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="E27" s="17" t="n">
+      <c r="E27" s="18" t="n">
         <v>180</v>
       </c>
-      <c r="F27" s="18" t="n">
+      <c r="F27" s="19" t="n">
         <f aca="false">C27-E27</f>
         <v>20</v>
       </c>
-      <c r="G27" s="17" t="n">
+      <c r="G27" s="18" t="n">
         <v>90</v>
       </c>
-      <c r="H27" s="18" t="n">
+      <c r="H27" s="19" t="n">
         <f aca="false">E27*G27</f>
         <v>16200</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="3" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="B28" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="C28" s="17" t="n">
+      <c r="C28" s="18" t="n">
         <v>100</v>
       </c>
-      <c r="D28" s="5"/>
-      <c r="E28" s="17" t="n">
+      <c r="D28" s="6"/>
+      <c r="E28" s="18" t="n">
         <v>90</v>
       </c>
-      <c r="F28" s="18" t="n">
+      <c r="F28" s="19" t="n">
         <f aca="false">C28-E28</f>
         <v>10</v>
       </c>
-      <c r="G28" s="17" t="n">
+      <c r="G28" s="18" t="n">
         <v>90</v>
       </c>
-      <c r="H28" s="18" t="n">
+      <c r="H28" s="19" t="n">
         <f aca="false">E28*G28</f>
         <v>8100</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="B29" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="C29" s="17" t="n">
+      <c r="C29" s="18" t="n">
         <v>200</v>
       </c>
-      <c r="D29" s="5"/>
-      <c r="E29" s="17" t="n">
+      <c r="D29" s="6"/>
+      <c r="E29" s="18" t="n">
         <v>180</v>
       </c>
-      <c r="F29" s="18" t="n">
+      <c r="F29" s="19" t="n">
         <f aca="false">C29-E29</f>
         <v>20</v>
       </c>
-      <c r="G29" s="17" t="n">
+      <c r="G29" s="18" t="n">
         <v>110</v>
       </c>
-      <c r="H29" s="18" t="n">
+      <c r="H29" s="19" t="n">
         <f aca="false">E29*G29</f>
         <v>19800</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="3" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="B30" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="C30" s="17" t="n">
+      <c r="C30" s="18" t="n">
         <v>200</v>
       </c>
-      <c r="D30" s="5"/>
-      <c r="E30" s="17" t="n">
+      <c r="D30" s="6"/>
+      <c r="E30" s="18" t="n">
         <v>150</v>
       </c>
-      <c r="F30" s="18" t="n">
+      <c r="F30" s="19" t="n">
         <f aca="false">C30-E30</f>
         <v>50</v>
       </c>
-      <c r="G30" s="17" t="n">
+      <c r="G30" s="18" t="n">
         <v>270</v>
       </c>
-      <c r="H30" s="18" t="n">
+      <c r="H30" s="19" t="n">
         <f aca="false">E30*G30</f>
         <v>40500</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="3" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="B31" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="C31" s="17" t="n">
+      <c r="C31" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="D31" s="5" t="s">
+      <c r="D31" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="E31" s="17" t="n">
+      <c r="E31" s="18" t="n">
         <v>180</v>
       </c>
-      <c r="F31" s="18" t="n">
+      <c r="F31" s="19" t="n">
         <f aca="false">C31-E31</f>
         <v>120</v>
       </c>
-      <c r="G31" s="17" t="n">
+      <c r="G31" s="18" t="n">
         <v>120</v>
       </c>
-      <c r="H31" s="18" t="n">
+      <c r="H31" s="19" t="n">
         <f aca="false">E31*G31</f>
         <v>21600</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="3" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="B32" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="C32" s="17" t="n">
+      <c r="C32" s="18" t="n">
         <v>120</v>
       </c>
-      <c r="D32" s="5"/>
-      <c r="E32" s="17" t="n">
+      <c r="D32" s="6"/>
+      <c r="E32" s="18" t="n">
         <v>100</v>
       </c>
-      <c r="F32" s="18" t="n">
+      <c r="F32" s="19" t="n">
         <f aca="false">C32-E32</f>
         <v>20</v>
       </c>
-      <c r="G32" s="17" t="n">
+      <c r="G32" s="18" t="n">
         <v>200</v>
       </c>
-      <c r="H32" s="18" t="n">
+      <c r="H32" s="19" t="n">
         <f aca="false">E32*G32</f>
         <v>20000</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="B33" s="3" t="s">
+      <c r="B33" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="C33" s="17" t="n">
+      <c r="C33" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="D33" s="5"/>
-      <c r="E33" s="17" t="n">
+      <c r="D33" s="6"/>
+      <c r="E33" s="18" t="n">
         <v>70</v>
       </c>
-      <c r="F33" s="18" t="n">
+      <c r="F33" s="19" t="n">
         <f aca="false">C33-E33</f>
         <v>10</v>
       </c>
-      <c r="G33" s="17" t="n">
+      <c r="G33" s="18" t="n">
         <v>100</v>
       </c>
-      <c r="H33" s="18" t="n">
+      <c r="H33" s="19" t="n">
         <f aca="false">E33*G33</f>
         <v>7000</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="3" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="B34" s="3" t="s">
+      <c r="B34" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="C34" s="17" t="n">
+      <c r="C34" s="18" t="n">
         <v>400</v>
       </c>
-      <c r="D34" s="5" t="s">
+      <c r="D34" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="E34" s="17" t="n">
+      <c r="E34" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="F34" s="18" t="n">
+      <c r="F34" s="19" t="n">
         <f aca="false">C34-E34</f>
         <v>100</v>
       </c>
-      <c r="G34" s="17" t="n">
+      <c r="G34" s="18" t="n">
         <v>150</v>
       </c>
-      <c r="H34" s="18" t="n">
+      <c r="H34" s="19" t="n">
         <f aca="false">E34*G34</f>
         <v>45000</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="19"/>
-      <c r="B35" s="20" t="s">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="20"/>
+      <c r="B35" s="21" t="s">
         <v>115</v>
       </c>
-      <c r="C35" s="20" t="n">
+      <c r="C35" s="21" t="n">
         <f aca="false">SUM(C3:C34)</f>
         <v>18240</v>
       </c>
-      <c r="D35" s="19"/>
-      <c r="E35" s="20" t="n">
+      <c r="D35" s="20"/>
+      <c r="E35" s="21" t="n">
         <f aca="false">SUM(E3:E34)</f>
-        <v>12970</v>
-      </c>
-      <c r="F35" s="20" t="n">
+        <v>13270</v>
+      </c>
+      <c r="F35" s="21" t="n">
         <f aca="false">SUM(F3:F34)</f>
-        <v>5270</v>
-      </c>
-      <c r="G35" s="19"/>
-      <c r="H35" s="20" t="n">
+        <v>4970</v>
+      </c>
+      <c r="G35" s="20"/>
+      <c r="H35" s="21" t="n">
         <f aca="false">SUM(H3:H34)</f>
-        <v>2028000</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="6" t="s">
+        <v>2073000</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="B37" s="15"/>
-      <c r="C37" s="21" t="n">
+      <c r="B37" s="16"/>
+      <c r="C37" s="22" t="n">
         <f aca="false">C35</f>
         <v>18240</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="6" t="s">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="B38" s="15"/>
-      <c r="C38" s="21" t="n">
+      <c r="B38" s="16"/>
+      <c r="C38" s="22" t="n">
         <f aca="false">E35</f>
-        <v>12970</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="6" t="s">
+        <v>13270</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="B39" s="15"/>
-      <c r="C39" s="21" t="n">
+      <c r="B39" s="16"/>
+      <c r="C39" s="22" t="n">
         <f aca="false">F35</f>
-        <v>5270</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="6" t="s">
+        <v>4970</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B40" s="15"/>
-      <c r="C40" s="22" t="n">
+      <c r="B40" s="16"/>
+      <c r="C40" s="23" t="n">
         <f aca="false">F35/C35</f>
-        <v>0.288925438596491</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="6" t="s">
+        <v>0.272478070175439</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="B41" s="15"/>
-      <c r="C41" s="21" t="n">
+      <c r="B41" s="16"/>
+      <c r="C41" s="22" t="n">
         <f aca="false">H35/E35</f>
-        <v>156.360832690825</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="16" t="s">
+        <v>156.21703089676</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="17" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="16" t="s">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="17" t="s">
         <v>121</v>
       </c>
     </row>

</xml_diff>